<commit_message>
Benchmark confidence tables: standardized log CIO age
The age interaction now uses log_cio_age standardized over the Table III
sample (mean 3.950, sd 0.174), in both the fye1 and fy versions.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qpw2BayLmQibPr7ZExRA1m
</commit_message>
<xml_diff>
--- a/referee_response/time_to_departure/benchmark_gradeA_tables.xlsx
+++ b/referee_response/time_to_departure/benchmark_gradeA_tables.xlsx
@@ -115,7 +115,7 @@
     <t xml:space="preserve">Interaction Specification: Peer- and Benchmark-Adjusted Returns by Benchmark Confidence</t>
   </si>
   <si>
-    <t xml:space="preserve">This table repeats the interaction specification of xsec_interactions_fye1.xlsx (all Table III controls, fiscal-year-end date fixed effects, Conflicted CIO interacted with X). Panel A uses Peer-Adjusted Return, for all plan-years and for the plan-years that also have the grade-A benchmark-adjusted return; Panel B uses Benchmark-Adjusted Return for three versions of the policy benchmark. Benchmark-Adjusted Return is the plan's return minus its policy benchmark return. 'Reported + inferred grade A/B' uses the benchmark return reported in the plan's financial report or, where none is stated, an inferred value graded A or B (the version in the earlier tables). 'Reported + inferred grade A only' drops the inferred values graded B (28 plan-years, 10 of them conflicted). 'Reported benchmarks only' drops all inferred values. For binary X, Conflicted CIO is the effect when X = 0 and the italic row gives the effect when X = 1. Continuous X (log pay, relative pay filled within spell, log CIO age) is centered at its regression-sample mean, so Conflicted CIO is the effect at average X, and the italic rows give the effect at the 25th and 75th percentiles. Log CIO Age is the paper's log_cio_age, ln(1 + age); that column drops the lagged log CIO age control. The standard errors are double clustered by plan and year. Coefficients marked with ***, **, and * are significant at the 1%, 5%, and 10% level, respectively.</t>
+    <t xml:space="preserve">This table repeats the interaction specification of xsec_interactions_fye1.xlsx (all Table III controls, fiscal-year-end date fixed effects, Conflicted CIO interacted with X). Panel A uses Peer-Adjusted Return, for all plan-years and for the plan-years that also have the grade-A benchmark-adjusted return; Panel B uses Benchmark-Adjusted Return for three versions of the policy benchmark. Benchmark-Adjusted Return is the plan's return minus its policy benchmark return. 'Reported + inferred grade A/B' uses the benchmark return reported in the plan's financial report or, where none is stated, an inferred value graded A or B (the version in the earlier tables). 'Reported + inferred grade A only' drops the inferred values graded B (28 plan-years, 10 of them conflicted). 'Reported benchmarks only' drops all inferred values. For binary X, Conflicted CIO is the effect when X = 0 and the italic row gives the effect when X = 1. Continuous X (log pay, relative pay filled within spell, standardized log CIO age) is centered at its regression-sample mean, so Conflicted CIO is the effect at average X, and the italic rows give the effect at the 25th and 75th percentiles. Log CIO Age (std.) is the paper's log_cio_age, ln(1 + age), standardized over the Table III sample (mean 3.950, standard deviation 0.174), so its interaction is the change in the effect of conflict for a one-standard-deviation increase in log age, about 10 years at the mean age of 52; that column drops the lagged log CIO age control. The standard errors are double clustered by plan and year. Coefficients marked with ***, **, and * are significant at the 1%, 5%, and 10% level, respectively.</t>
   </si>
   <si>
     <t xml:space="preserve">X = Underpaid</t>
@@ -142,7 +142,7 @@
     <t xml:space="preserve">X = Relative CIO Pay (filled)</t>
   </si>
   <si>
-    <t xml:space="preserve">X = Log CIO Age</t>
+    <t xml:space="preserve">X = Log CIO Age (std.)</t>
   </si>
   <si>
     <t xml:space="preserve">Conflicted CIO x X</t>
@@ -265,7 +265,7 @@
     <t xml:space="preserve">Relative CIO Pay (filled)</t>
   </si>
   <si>
-    <t xml:space="preserve">Log CIO Age</t>
+    <t xml:space="preserve">Log CIO Age (std.)</t>
   </si>
 </sst>
 </file>
@@ -847,7 +847,7 @@
         <v>0.0811821814459482</v>
       </c>
       <c r="E11" s="10" t="n">
-        <v>0.095642067766866</v>
+        <v>0.0956420677668662</v>
       </c>
       <c r="F11" s="10" t="n">
         <v>0.0555249057485127</v>
@@ -976,7 +976,7 @@
         <v>0.0825523730429406</v>
       </c>
       <c r="E18" s="10" t="n">
-        <v>0.104185873254466</v>
+        <v>0.104185873254457</v>
       </c>
       <c r="F18" s="10" t="n">
         <v>0.0674388145832005</v>
@@ -1110,7 +1110,7 @@
         <v>0.0207392892531291</v>
       </c>
       <c r="E26" s="10" t="n">
-        <v>0.122153932551764</v>
+        <v>0.122153932551761</v>
       </c>
       <c r="F26" s="10" t="n">
         <v>0.124841777309274</v>
@@ -1239,7 +1239,7 @@
         <v>0.021627094632006</v>
       </c>
       <c r="E33" s="10" t="n">
-        <v>0.121740184553309</v>
+        <v>0.121740184553304</v>
       </c>
       <c r="F33" s="10" t="n">
         <v>0.126079127494547</v>
@@ -1368,7 +1368,7 @@
         <v>0.0160513439245875</v>
       </c>
       <c r="E40" s="10" t="n">
-        <v>0.108381335691557</v>
+        <v>0.108381335691552</v>
       </c>
       <c r="F40" s="10" t="n">
         <v>0.117176365151909</v>
@@ -1492,7 +1492,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="168" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="181.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>30</v>
       </c>
@@ -1663,7 +1663,7 @@
       </c>
       <c r="J9" s="8" t="str">
         <f aca="false">IF(Estimates!I51="","",TEXT(Estimates!E51,"0.000")&amp;IF(Estimates!I51&lt;0.01,"***",IF(Estimates!I51&lt;0.05,"**",IF(Estimates!I51&lt;0.1,"*",""))))</f>
-        <v>2.206*</v>
+        <v>0.385*</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1742,7 +1742,7 @@
       </c>
       <c r="J11" s="8" t="str">
         <f aca="false">IF(Estimates!I60="","",TEXT(Estimates!E60,"0.000")&amp;IF(Estimates!I60&lt;0.01,"***",IF(Estimates!I60&lt;0.05,"**",IF(Estimates!I60&lt;0.1,"*",""))))</f>
-        <v>-0.784</v>
+        <v>-0.137</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1780,7 +1780,7 @@
       </c>
       <c r="J12" s="8" t="str">
         <f aca="false">IF(Estimates!H60="","","("&amp;TEXT(Estimates!H60,"0.00")&amp;")")</f>
-        <v>(-1.14)</v>
+        <v>(-1.13)</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2075,7 +2075,7 @@
       </c>
       <c r="J27" s="8" t="str">
         <f aca="false">IF(Estimates!H81="","","("&amp;TEXT(Estimates!H81,"0.00")&amp;")")</f>
-        <v>(-1.63)</v>
+        <v>(-1.62)</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2116,7 +2116,7 @@
       </c>
       <c r="J28" s="8" t="str">
         <f aca="false">IF(Estimates!I90="","",TEXT(Estimates!E90,"0.000")&amp;IF(Estimates!I90&lt;0.01,"***",IF(Estimates!I90&lt;0.05,"**",IF(Estimates!I90&lt;0.1,"*",""))))</f>
-        <v>2.697**</v>
+        <v>0.470**</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2154,7 +2154,7 @@
       </c>
       <c r="J29" s="8" t="str">
         <f aca="false">IF(Estimates!H90="","","("&amp;TEXT(Estimates!H90,"0.00")&amp;")")</f>
-        <v>(2.23)</v>
+        <v>(2.22)</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2195,7 +2195,7 @@
       </c>
       <c r="J30" s="8" t="str">
         <f aca="false">IF(Estimates!I99="","",TEXT(Estimates!E99,"0.000")&amp;IF(Estimates!I99&lt;0.01,"***",IF(Estimates!I99&lt;0.05,"**",IF(Estimates!I99&lt;0.1,"*",""))))</f>
-        <v>-1.059</v>
+        <v>-0.185</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2233,7 +2233,7 @@
       </c>
       <c r="J31" s="8" t="str">
         <f aca="false">IF(Estimates!H99="","","("&amp;TEXT(Estimates!H99,"0.00")&amp;")")</f>
-        <v>(-1.38)</v>
+        <v>(-1.35)</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2319,7 +2319,7 @@
       </c>
       <c r="J36" s="14" t="str">
         <f aca="false">IF(Estimates!H108="","","("&amp;TEXT(Estimates!H108,"0.00")&amp;")")</f>
-        <v>(-2.46)</v>
+        <v>(-2.45)</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2574,7 +2574,7 @@
       </c>
       <c r="J48" s="8" t="str">
         <f aca="false">IF(Estimates!I129="","",TEXT(Estimates!E129,"0.000")&amp;IF(Estimates!I129&lt;0.01,"***",IF(Estimates!I129&lt;0.05,"**",IF(Estimates!I129&lt;0.1,"*",""))))</f>
-        <v>1.068</v>
+        <v>0.186</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2612,7 +2612,7 @@
       </c>
       <c r="J49" s="8" t="str">
         <f aca="false">IF(Estimates!H129="","","("&amp;TEXT(Estimates!H129,"0.00")&amp;")")</f>
-        <v>(1.50)</v>
+        <v>(1.49)</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2653,7 +2653,7 @@
       </c>
       <c r="J50" s="8" t="str">
         <f aca="false">IF(Estimates!I138="","",TEXT(Estimates!E138,"0.000")&amp;IF(Estimates!I138&lt;0.01,"***",IF(Estimates!I138&lt;0.05,"**",IF(Estimates!I138&lt;0.1,"*",""))))</f>
-        <v>-1.098</v>
+        <v>-0.191</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="J67" s="8" t="str">
         <f aca="false">IF(Estimates!I168="","",TEXT(Estimates!E168,"0.000")&amp;IF(Estimates!I168&lt;0.01,"***",IF(Estimates!I168&lt;0.05,"**",IF(Estimates!I168&lt;0.1,"*",""))))</f>
-        <v>0.977</v>
+        <v>0.170</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3106,7 +3106,7 @@
       </c>
       <c r="J69" s="8" t="str">
         <f aca="false">IF(Estimates!I177="","",TEXT(Estimates!E177,"0.000")&amp;IF(Estimates!I177&lt;0.01,"***",IF(Estimates!I177&lt;0.05,"**",IF(Estimates!I177&lt;0.1,"*",""))))</f>
-        <v>-1.087</v>
+        <v>-0.189</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3144,7 +3144,7 @@
       </c>
       <c r="J70" s="8" t="str">
         <f aca="false">IF(Estimates!H177="","","("&amp;TEXT(Estimates!H177,"0.00")&amp;")")</f>
-        <v>(-1.62)</v>
+        <v>(-1.61)</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3439,7 +3439,7 @@
       </c>
       <c r="J85" s="8" t="str">
         <f aca="false">IF(Estimates!H198="","","("&amp;TEXT(Estimates!H198,"0.00")&amp;")")</f>
-        <v>(-2.21)</v>
+        <v>(-2.22)</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3480,7 +3480,7 @@
       </c>
       <c r="J86" s="8" t="str">
         <f aca="false">IF(Estimates!I207="","",TEXT(Estimates!E207,"0.000")&amp;IF(Estimates!I207&lt;0.01,"***",IF(Estimates!I207&lt;0.05,"**",IF(Estimates!I207&lt;0.1,"*",""))))</f>
-        <v>0.764</v>
+        <v>0.133</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3518,7 +3518,7 @@
       </c>
       <c r="J87" s="8" t="str">
         <f aca="false">IF(Estimates!H207="","","("&amp;TEXT(Estimates!H207,"0.00")&amp;")")</f>
-        <v>(1.12)</v>
+        <v>(1.11)</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3559,7 +3559,7 @@
       </c>
       <c r="J88" s="8" t="str">
         <f aca="false">IF(Estimates!I216="","",TEXT(Estimates!E216,"0.000")&amp;IF(Estimates!I216&lt;0.01,"***",IF(Estimates!I216&lt;0.05,"**",IF(Estimates!I216&lt;0.1,"*",""))))</f>
-        <v>-0.757</v>
+        <v>-0.132</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="J89" s="8" t="str">
         <f aca="false">IF(Estimates!H216="","","("&amp;TEXT(Estimates!H216,"0.00")&amp;")")</f>
-        <v>(-1.22)</v>
+        <v>(-1.21)</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="J94" s="14" t="str">
         <f aca="false">IF(Estimates!H225="","","("&amp;TEXT(Estimates!H225,"0.00")&amp;")")</f>
-        <v>(-2.97)</v>
+        <v>(-2.94)</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3714,7 +3714,7 @@
       </c>
       <c r="J96" s="14" t="str">
         <f aca="false">IF(Estimates!H228="","","("&amp;TEXT(Estimates!H228,"0.00")&amp;")")</f>
-        <v>(-1.21)</v>
+        <v>(-1.22)</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4084,21 +4084,21 @@
         <v>66</v>
       </c>
       <c r="E7" s="22" t="n">
-        <v>-0.69792191317879</v>
+        <v>-0.697921913178826</v>
       </c>
       <c r="F7" s="22" t="n">
-        <v>0.293738442045888</v>
+        <v>0.29373848060631</v>
       </c>
       <c r="G7" s="23" t="n">
         <v>19</v>
       </c>
       <c r="H7" s="24" t="n">
         <f aca="false">IF(F7&gt;0,E7/F7,"")</f>
-        <v>-2.37599787184056</v>
+        <v>-2.37599755993234</v>
       </c>
       <c r="I7" s="24" t="n">
         <f aca="false">IF(H7="","",TDIST(ABS(H7),G7-1,2))</f>
-        <v>0.0288095820574215</v>
+        <v>0.0288096004414067</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4270,21 +4270,21 @@
         <v>66</v>
       </c>
       <c r="E13" s="22" t="n">
-        <v>-0.642193007103207</v>
+        <v>-0.642193007103368</v>
       </c>
       <c r="F13" s="22" t="n">
-        <v>0.284269769945482</v>
+        <v>0.284269738993169</v>
       </c>
       <c r="G13" s="23" t="n">
         <v>19</v>
       </c>
       <c r="H13" s="24" t="n">
         <f aca="false">IF(F13&gt;0,E13/F13,"")</f>
-        <v>-2.25909707960283</v>
+        <v>-2.25909732558202</v>
       </c>
       <c r="I13" s="24" t="n">
         <f aca="false">IF(H13="","",TDIST(ABS(H13),G13-1,2))</f>
-        <v>0.036521229486758</v>
+        <v>0.0365212114168489</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4456,21 +4456,21 @@
         <v>66</v>
       </c>
       <c r="E19" s="22" t="n">
-        <v>-0.411441281849598</v>
+        <v>-0.411441281849561</v>
       </c>
       <c r="F19" s="22" t="n">
-        <v>0.191635803827689</v>
+        <v>0.191635803149997</v>
       </c>
       <c r="G19" s="23" t="n">
         <v>19</v>
       </c>
       <c r="H19" s="24" t="n">
         <f aca="false">IF(F19&gt;0,E19/F19,"")</f>
-        <v>-2.14699588297994</v>
+        <v>-2.14699589057227</v>
       </c>
       <c r="I19" s="24" t="n">
         <f aca="false">IF(H19="","",TDIST(ABS(H19),G19-1,2))</f>
-        <v>0.0456671756972536</v>
+        <v>0.0456671750124047</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4642,21 +4642,21 @@
         <v>66</v>
       </c>
       <c r="E25" s="22" t="n">
-        <v>-0.387587771011477</v>
+        <v>-0.387587771011609</v>
       </c>
       <c r="F25" s="22" t="n">
-        <v>0.185144671149296</v>
+        <v>0.185144692631368</v>
       </c>
       <c r="G25" s="23" t="n">
         <v>19</v>
       </c>
       <c r="H25" s="24" t="n">
         <f aca="false">IF(F25&gt;0,E25/F25,"")</f>
-        <v>-2.09343195569985</v>
+        <v>-2.09343171280267</v>
       </c>
       <c r="I25" s="24" t="n">
         <f aca="false">IF(H25="","",TDIST(ABS(H25),G25-1,2))</f>
-        <v>0.0507387097464345</v>
+        <v>0.0507387338620792</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4828,21 +4828,21 @@
         <v>66</v>
       </c>
       <c r="E31" s="22" t="n">
-        <v>-0.333186779111117</v>
+        <v>-0.33318677911114</v>
       </c>
       <c r="F31" s="22" t="n">
-        <v>0.156813610430477</v>
+        <v>0.156813617007179</v>
       </c>
       <c r="G31" s="23" t="n">
         <v>19</v>
       </c>
       <c r="H31" s="24" t="n">
         <f aca="false">IF(F31&gt;0,E31/F31,"")</f>
-        <v>-2.1247312538527</v>
+        <v>-2.12473116474245</v>
       </c>
       <c r="I31" s="24" t="n">
         <f aca="false">IF(H31="","",TDIST(ABS(H31),G31-1,2))</f>
-        <v>0.047716302310565</v>
+        <v>0.0477163106769723</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5169,21 +5169,21 @@
         <v>10</v>
       </c>
       <c r="E42" s="22" t="n">
-        <v>-0.293307954355725</v>
+        <v>-0.293307954355724</v>
       </c>
       <c r="F42" s="22" t="n">
-        <v>0.14258132105269</v>
+        <v>0.142609173177447</v>
       </c>
       <c r="G42" s="23" t="n">
         <v>19</v>
       </c>
       <c r="H42" s="24" t="n">
         <f aca="false">IF(F42&gt;0,E42/F42,"")</f>
-        <v>-2.057127484794</v>
+        <v>-2.05672571981582</v>
       </c>
       <c r="I42" s="24" t="n">
         <f aca="false">IF(H42="","",TDIST(ABS(H42),G42-1,2))</f>
-        <v>0.0544615186842412</v>
+        <v>0.054504065935473</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5448,21 +5448,21 @@
         <v>40</v>
       </c>
       <c r="E51" s="22" t="n">
-        <v>2.20641163750183</v>
+        <v>0.384576834565827</v>
       </c>
       <c r="F51" s="22" t="n">
-        <v>1.06033444628367</v>
+        <v>0.184878922222022</v>
       </c>
       <c r="G51" s="23" t="n">
         <v>19</v>
       </c>
       <c r="H51" s="24" t="n">
         <f aca="false">IF(F51&gt;0,E51/F51,"")</f>
-        <v>2.08086386822102</v>
+        <v>2.08015510877972</v>
       </c>
       <c r="I51" s="24" t="n">
         <f aca="false">IF(H51="","",TDIST(ABS(H51),G51-1,2))</f>
-        <v>0.052000532717402</v>
+        <v>0.0520725322381767</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5727,21 +5727,21 @@
         <v>41</v>
       </c>
       <c r="E60" s="22" t="n">
-        <v>-0.784028424071975</v>
+        <v>-0.136655900655339</v>
       </c>
       <c r="F60" s="22" t="n">
-        <v>0.684771349559568</v>
+        <v>0.120492687637552</v>
       </c>
       <c r="G60" s="23" t="n">
         <v>19</v>
       </c>
       <c r="H60" s="24" t="n">
         <f aca="false">IF(F60&gt;0,E60/F60,"")</f>
-        <v>-1.144949222213</v>
+        <v>-1.13414268811404</v>
       </c>
       <c r="I60" s="24" t="n">
         <f aca="false">IF(H60="","",TDIST(ABS(H60),G60-1,2))</f>
-        <v>0.267226498788926</v>
+        <v>0.27161382284148</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6009,18 +6009,18 @@
         <v>-0.540779013200599</v>
       </c>
       <c r="F69" s="22" t="n">
-        <v>0.198424242668066</v>
+        <v>0.198428471405626</v>
       </c>
       <c r="G69" s="23" t="n">
         <v>19</v>
       </c>
       <c r="H69" s="24" t="n">
         <f aca="false">IF(F69&gt;0,E69/F69,"")</f>
-        <v>-2.72536765633644</v>
+        <v>-2.72530957563616</v>
       </c>
       <c r="I69" s="24" t="n">
         <f aca="false">IF(H69="","",TDIST(ABS(H69),G69-1,2))</f>
-        <v>0.0138823105159941</v>
+        <v>0.0138840270479958</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6099,21 +6099,21 @@
         <v>44</v>
       </c>
       <c r="E72" s="22" t="n">
-        <v>-0.039063419130387</v>
+        <v>-0.039063419130385</v>
       </c>
       <c r="F72" s="22" t="n">
-        <v>0.173852624332739</v>
+        <v>0.173951697308515</v>
       </c>
       <c r="G72" s="23" t="n">
         <v>19</v>
       </c>
       <c r="H72" s="24" t="n">
         <f aca="false">IF(F72&gt;0,E72/F72,"")</f>
-        <v>-0.224692720517253</v>
+        <v>-0.224564748345648</v>
       </c>
       <c r="I72" s="24" t="n">
         <f aca="false">IF(H72="","",TDIST(ABS(H72),G72-1,2))</f>
-        <v>0.824749284447918</v>
+        <v>0.824847341190403</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6381,18 +6381,18 @@
         <v>-0.238402609294629</v>
       </c>
       <c r="F81" s="22" t="n">
-        <v>0.146603787013093</v>
+        <v>0.147137656131034</v>
       </c>
       <c r="G81" s="23" t="n">
         <v>19</v>
       </c>
       <c r="H81" s="24" t="n">
         <f aca="false">IF(F81&gt;0,E81/F81,"")</f>
-        <v>-1.62616951548009</v>
+        <v>-1.62026917896747</v>
       </c>
       <c r="I81" s="24" t="n">
         <f aca="false">IF(H81="","",TDIST(ABS(H81),G81-1,2))</f>
-        <v>0.121292780409653</v>
+        <v>0.122560920188969</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6657,21 +6657,21 @@
         <v>40</v>
       </c>
       <c r="E90" s="22" t="n">
-        <v>2.69671336042971</v>
+        <v>0.47003626624253</v>
       </c>
       <c r="F90" s="22" t="n">
-        <v>1.21185092840965</v>
+        <v>0.211344374863824</v>
       </c>
       <c r="G90" s="23" t="n">
         <v>19</v>
       </c>
       <c r="H90" s="24" t="n">
         <f aca="false">IF(F90&gt;0,E90/F90,"")</f>
-        <v>2.22528472538177</v>
+        <v>2.22403017135133</v>
       </c>
       <c r="I90" s="24" t="n">
         <f aca="false">IF(H90="","",TDIST(ABS(H90),G90-1,2))</f>
-        <v>0.0390845711299189</v>
+        <v>0.0391827946841477</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6936,21 +6936,21 @@
         <v>41</v>
       </c>
       <c r="E99" s="22" t="n">
-        <v>-1.05853028736798</v>
+        <v>-0.184501486616952</v>
       </c>
       <c r="F99" s="22" t="n">
-        <v>0.769131953100291</v>
+        <v>0.137111943522795</v>
       </c>
       <c r="G99" s="23" t="n">
         <v>19</v>
       </c>
       <c r="H99" s="24" t="n">
         <f aca="false">IF(F99&gt;0,E99/F99,"")</f>
-        <v>-1.37626617006504</v>
+        <v>-1.34562666006028</v>
       </c>
       <c r="I99" s="24" t="n">
         <f aca="false">IF(H99="","",TDIST(ABS(H99),G99-1,2))</f>
-        <v>0.1856207878382</v>
+        <v>0.195129475071542</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7215,21 +7215,21 @@
         <v>43</v>
       </c>
       <c r="E108" s="22" t="n">
-        <v>-0.533399815068965</v>
+        <v>-0.533399815068966</v>
       </c>
       <c r="F108" s="22" t="n">
-        <v>0.216769186904159</v>
+        <v>0.217409745408931</v>
       </c>
       <c r="G108" s="23" t="n">
         <v>19</v>
       </c>
       <c r="H108" s="24" t="n">
         <f aca="false">IF(F108&gt;0,E108/F108,"")</f>
-        <v>-2.46068097909505</v>
+        <v>-2.45343102750836</v>
       </c>
       <c r="I108" s="24" t="n">
         <f aca="false">IF(H108="","",TDIST(ABS(H108),G108-1,2))</f>
-        <v>0.0242031058760117</v>
+        <v>0.0245686624361504</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7308,21 +7308,21 @@
         <v>44</v>
       </c>
       <c r="E111" s="22" t="n">
-        <v>0.0798054104060772</v>
+        <v>0.0798054104060767</v>
       </c>
       <c r="F111" s="22" t="n">
-        <v>0.182742656746656</v>
+        <v>0.182935301745309</v>
       </c>
       <c r="G111" s="23" t="n">
         <v>19</v>
       </c>
       <c r="H111" s="24" t="n">
         <f aca="false">IF(F111&gt;0,E111/F111,"")</f>
-        <v>0.436709260042745</v>
+        <v>0.436249371470059</v>
       </c>
       <c r="I111" s="24" t="n">
         <f aca="false">IF(H111="","",TDIST(ABS(H111),G111-1,2))</f>
-        <v>0.667515805175875</v>
+        <v>0.667843240426049</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7587,21 +7587,21 @@
         <v>10</v>
       </c>
       <c r="E120" s="22" t="n">
-        <v>-0.349407805307186</v>
+        <v>-0.349407805307187</v>
       </c>
       <c r="F120" s="22" t="n">
-        <v>0.144832605118093</v>
+        <v>0.1448261917769</v>
       </c>
       <c r="G120" s="23" t="n">
         <v>19</v>
       </c>
       <c r="H120" s="24" t="n">
         <f aca="false">IF(F120&gt;0,E120/F120,"")</f>
-        <v>-2.41249409980776</v>
+        <v>-2.41260093233301</v>
       </c>
       <c r="I120" s="24" t="n">
         <f aca="false">IF(H120="","",TDIST(ABS(H120),G120-1,2))</f>
-        <v>0.0267319029643468</v>
+        <v>0.0267260322613237</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7866,21 +7866,21 @@
         <v>40</v>
       </c>
       <c r="E129" s="22" t="n">
-        <v>1.06763672412182</v>
+        <v>0.186088735596897</v>
       </c>
       <c r="F129" s="22" t="n">
-        <v>0.713378665232936</v>
+        <v>0.124605699366767</v>
       </c>
       <c r="G129" s="23" t="n">
         <v>19</v>
       </c>
       <c r="H129" s="24" t="n">
         <f aca="false">IF(F129&gt;0,E129/F129,"")</f>
-        <v>1.49659188892789</v>
+        <v>1.49342073871887</v>
       </c>
       <c r="I129" s="24" t="n">
         <f aca="false">IF(H129="","",TDIST(ABS(H129),G129-1,2))</f>
-        <v>0.151828498515247</v>
+        <v>0.152649280269266</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8145,21 +8145,21 @@
         <v>41</v>
       </c>
       <c r="E138" s="22" t="n">
-        <v>-1.09773747829353</v>
+        <v>-0.191335287310388</v>
       </c>
       <c r="F138" s="22" t="n">
-        <v>0.676016329731197</v>
+        <v>0.117862236607252</v>
       </c>
       <c r="G138" s="23" t="n">
         <v>19</v>
       </c>
       <c r="H138" s="24" t="n">
         <f aca="false">IF(F138&gt;0,E138/F138,"")</f>
-        <v>-1.62383278334418</v>
+        <v>-1.62338076060755</v>
       </c>
       <c r="I138" s="24" t="n">
         <f aca="false">IF(H138="","",TDIST(ABS(H138),G138-1,2))</f>
-        <v>0.121793669309044</v>
+        <v>0.121890764596971</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8427,18 +8427,18 @@
         <v>-0.466194797310107</v>
       </c>
       <c r="F147" s="22" t="n">
-        <v>0.143284706885311</v>
+        <v>0.143254597996585</v>
       </c>
       <c r="G147" s="23" t="n">
         <v>19</v>
       </c>
       <c r="H147" s="24" t="n">
         <f aca="false">IF(F147&gt;0,E147/F147,"")</f>
-        <v>-3.25362564815283</v>
+        <v>-3.25430948695428</v>
       </c>
       <c r="I147" s="24" t="n">
         <f aca="false">IF(H147="","",TDIST(ABS(H147),G147-1,2))</f>
-        <v>0.00441004144016498</v>
+        <v>0.00440340150243833</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8517,21 +8517,21 @@
         <v>44</v>
       </c>
       <c r="E150" s="22" t="n">
-        <v>-0.223425051089754</v>
+        <v>-0.223425051089755</v>
       </c>
       <c r="F150" s="22" t="n">
-        <v>0.187384101957315</v>
+        <v>0.187553458215477</v>
       </c>
       <c r="G150" s="23" t="n">
         <v>19</v>
       </c>
       <c r="H150" s="24" t="n">
         <f aca="false">IF(F150&gt;0,E150/F150,"")</f>
-        <v>-1.19233728345134</v>
+        <v>-1.19126063158519</v>
       </c>
       <c r="I150" s="24" t="n">
         <f aca="false">IF(H150="","",TDIST(ABS(H150),G150-1,2))</f>
-        <v>0.248611327611516</v>
+        <v>0.249023070406589</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8799,18 +8799,18 @@
         <v>-0.33346924587246</v>
       </c>
       <c r="F159" s="22" t="n">
-        <v>0.148100482687894</v>
+        <v>0.148061344592865</v>
       </c>
       <c r="G159" s="23" t="n">
         <v>19</v>
       </c>
       <c r="H159" s="24" t="n">
         <f aca="false">IF(F159&gt;0,E159/F159,"")</f>
-        <v>-2.25164185707086</v>
+        <v>-2.25223704937588</v>
       </c>
       <c r="I159" s="24" t="n">
         <f aca="false">IF(H159="","",TDIST(ABS(H159),G159-1,2))</f>
-        <v>0.0370727066860094</v>
+        <v>0.0370283983883391</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9075,21 +9075,21 @@
         <v>40</v>
       </c>
       <c r="E168" s="22" t="n">
-        <v>0.977223734924737</v>
+        <v>0.170329780831587</v>
       </c>
       <c r="F168" s="22" t="n">
-        <v>0.697004542367146</v>
+        <v>0.12185521160248</v>
       </c>
       <c r="G168" s="23" t="n">
         <v>19</v>
       </c>
       <c r="H168" s="24" t="n">
         <f aca="false">IF(F168&gt;0,E168/F168,"")</f>
-        <v>1.40203352420907</v>
+        <v>1.39780464529692</v>
       </c>
       <c r="I168" s="24" t="n">
         <f aca="false">IF(H168="","",TDIST(ABS(H168),G168-1,2))</f>
-        <v>0.1779150045409</v>
+        <v>0.179161662717305</v>
       </c>
     </row>
     <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9354,21 +9354,21 @@
         <v>41</v>
       </c>
       <c r="E177" s="22" t="n">
-        <v>-1.08720014472238</v>
+        <v>-0.189498633478131</v>
       </c>
       <c r="F177" s="22" t="n">
-        <v>0.672971951692254</v>
+        <v>0.117375932068108</v>
       </c>
       <c r="G177" s="23" t="n">
         <v>19</v>
       </c>
       <c r="H177" s="24" t="n">
         <f aca="false">IF(F177&gt;0,E177/F177,"")</f>
-        <v>-1.61552073899739</v>
+        <v>-1.61445903039282</v>
       </c>
       <c r="I177" s="24" t="n">
         <f aca="false">IF(H177="","",TDIST(ABS(H177),G177-1,2))</f>
-        <v>0.123589629811742</v>
+        <v>0.123820637488995</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9633,21 +9633,21 @@
         <v>43</v>
       </c>
       <c r="E186" s="22" t="n">
-        <v>-0.440369102360441</v>
+        <v>-0.440369102360442</v>
       </c>
       <c r="F186" s="22" t="n">
-        <v>0.142085353354917</v>
+        <v>0.142175084440911</v>
       </c>
       <c r="G186" s="23" t="n">
         <v>19</v>
       </c>
       <c r="H186" s="24" t="n">
         <f aca="false">IF(F186&gt;0,E186/F186,"")</f>
-        <v>-3.09932791777938</v>
+        <v>-3.09737183622678</v>
       </c>
       <c r="I186" s="24" t="n">
         <f aca="false">IF(H186="","",TDIST(ABS(H186),G186-1,2))</f>
-        <v>0.00618840984714248</v>
+        <v>0.00621494277343435</v>
       </c>
     </row>
     <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9729,18 +9729,18 @@
         <v>-0.218158351486051</v>
       </c>
       <c r="F189" s="22" t="n">
-        <v>0.191968290639688</v>
+        <v>0.192039601081895</v>
       </c>
       <c r="G189" s="23" t="n">
         <v>19</v>
       </c>
       <c r="H189" s="24" t="n">
         <f aca="false">IF(F189&gt;0,E189/F189,"")</f>
-        <v>-1.13642909857191</v>
+        <v>-1.13600710612296</v>
       </c>
       <c r="I189" s="24" t="n">
         <f aca="false">IF(H189="","",TDIST(ABS(H189),G189-1,2))</f>
-        <v>0.270681129271702</v>
+        <v>0.270853092870999</v>
       </c>
     </row>
     <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10008,18 +10008,18 @@
         <v>-0.323882701271995</v>
       </c>
       <c r="F198" s="22" t="n">
-        <v>0.14670773988722</v>
+        <v>0.145954332126848</v>
       </c>
       <c r="G198" s="23" t="n">
         <v>19</v>
       </c>
       <c r="H198" s="24" t="n">
         <f aca="false">IF(F198&gt;0,E198/F198,"")</f>
-        <v>-2.20767289797372</v>
+        <v>-2.21906877687269</v>
       </c>
       <c r="I198" s="24" t="n">
         <f aca="false">IF(H198="","",TDIST(ABS(H198),G198-1,2))</f>
-        <v>0.0404844232176984</v>
+        <v>0.0395734703201426</v>
       </c>
     </row>
     <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10284,21 +10284,21 @@
         <v>40</v>
       </c>
       <c r="E207" s="22" t="n">
-        <v>0.764280389179767</v>
+        <v>0.1332138245628</v>
       </c>
       <c r="F207" s="22" t="n">
-        <v>0.685136728236859</v>
+        <v>0.119995993515943</v>
       </c>
       <c r="G207" s="23" t="n">
         <v>19</v>
       </c>
       <c r="H207" s="24" t="n">
         <f aca="false">IF(F207&gt;0,E207/F207,"")</f>
-        <v>1.11551513395958</v>
+        <v>1.11015226975142</v>
       </c>
       <c r="I207" s="24" t="n">
         <f aca="false">IF(H207="","",TDIST(ABS(H207),G207-1,2))</f>
-        <v>0.279301607754385</v>
+        <v>0.281544416725914</v>
       </c>
     </row>
     <row r="208" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10563,21 +10563,21 @@
         <v>41</v>
       </c>
       <c r="E216" s="22" t="n">
-        <v>-0.756679243953135</v>
+        <v>-0.131888947409034</v>
       </c>
       <c r="F216" s="22" t="n">
-        <v>0.619701530488724</v>
+        <v>0.108838260675383</v>
       </c>
       <c r="G216" s="23" t="n">
         <v>19</v>
       </c>
       <c r="H216" s="24" t="n">
         <f aca="false">IF(F216&gt;0,E216/F216,"")</f>
-        <v>-1.22103820424065</v>
+        <v>-1.21178845187907</v>
       </c>
       <c r="I216" s="24" t="n">
         <f aca="false">IF(H216="","",TDIST(ABS(H216),G216-1,2))</f>
-        <v>0.237824959798012</v>
+        <v>0.24126139181854</v>
       </c>
     </row>
     <row r="217" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10842,21 +10842,21 @@
         <v>43</v>
       </c>
       <c r="E225" s="22" t="n">
-        <v>-0.392834428267741</v>
+        <v>-0.39283442826774</v>
       </c>
       <c r="F225" s="22" t="n">
-        <v>0.132200178189983</v>
+        <v>0.133419745026281</v>
       </c>
       <c r="G225" s="23" t="n">
         <v>19</v>
       </c>
       <c r="H225" s="24" t="n">
         <f aca="false">IF(F225&gt;0,E225/F225,"")</f>
-        <v>-2.971512093601</v>
+        <v>-2.94435001498737</v>
       </c>
       <c r="I225" s="24" t="n">
         <f aca="false">IF(H225="","",TDIST(ABS(H225),G225-1,2))</f>
-        <v>0.00817611172529997</v>
+        <v>0.00867218071127748</v>
       </c>
     </row>
     <row r="226" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10935,21 +10935,21 @@
         <v>44</v>
       </c>
       <c r="E228" s="22" t="n">
-        <v>-0.235135538954195</v>
+        <v>-0.235135538954196</v>
       </c>
       <c r="F228" s="22" t="n">
-        <v>0.194879366384004</v>
+        <v>0.192783972458412</v>
       </c>
       <c r="G228" s="23" t="n">
         <v>19</v>
       </c>
       <c r="H228" s="24" t="n">
         <f aca="false">IF(F228&gt;0,E228/F228,"")</f>
-        <v>-1.20656970164234</v>
+        <v>-1.2196840637513</v>
       </c>
       <c r="I228" s="24" t="n">
         <f aca="false">IF(H228="","",TDIST(ABS(H228),G228-1,2))</f>
-        <v>0.243216909515053</v>
+        <v>0.238325689667738</v>
       </c>
     </row>
   </sheetData>

</xml_diff>